<commit_message>
Updated map for paper
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/01_paper_IAEE/01_data_sheets_input/paper_paris_2025_input_production_europe_capacities.xlsx
+++ b/01_data/01_input_data/02_processed/01_paper_IAEE/01_data_sheets_input/paper_paris_2025_input_production_europe_capacities.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\01_paper_IAEE\01_data_sheets_input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://studentcbs-my.sharepoint.com/personal/mar_eco_cbs_dk/Documents/Desktop/hydrogen_grid/01_data/01_input_data/02_processed/01_paper_IAEE/01_data_sheets_input/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B41F561-B38A-4E02-A7B4-D63B1A86D5B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{61051CAB-F224-4792-AEE8-218AA7F2319D}"/>
+    <workbookView xWindow="-3840" yWindow="-17140" windowWidth="16300" windowHeight="15140" xr2:uid="{61051CAB-F224-4792-AEE8-218AA7F2319D}"/>
   </bookViews>
   <sheets>
     <sheet name="gas_production_GWh-a" sheetId="1" r:id="rId1"/>

</xml_diff>